<commit_message>
Add person scale and assumption-labelled indoor room sizing model
</commit_message>
<xml_diff>
--- a/reports/shareable_20261005/stakeholder/STAKEHOLDER_FUNDING.xlsx
+++ b/reports/shareable_20261005/stakeholder/STAKEHOLDER_FUNDING.xlsx
@@ -10,7 +10,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read me" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Milestones" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Claims" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Funding quotes" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Room scenarios" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Funding quotes" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Read me'!$A$1:$B$6</definedName>
@@ -19,8 +20,10 @@
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Milestones'!$1:$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Claims'!$A$1:$C$6</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Claims'!$1:$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Funding quotes'!$A$1:$M$16</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="3">'Funding quotes'!$1:$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Room scenarios'!$A$1:$H$5</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="3">'Room scenarios'!$1:$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Funding quotes'!$A$1:$M$16</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="4">'Funding quotes'!$1:$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -72,13 +75,19 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -815,6 +824,216 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
+  <dimension ref="A1:H5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14.95" customWidth="1" min="4" max="4"/>
+    <col width="55" customWidth="1" min="5" max="5"/>
+    <col width="55" customWidth="1" min="6" max="6"/>
+    <col width="55" customWidth="1" min="7" max="7"/>
+    <col width="25.35" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>ASSUMED area m2</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>ASSUMED height m</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>ASSUMED CADR m3/h</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Target fraction reduced</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Volume m3</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Ideal target minutes</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Required CADR for30 min</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="68" customHeight="1">
+      <c r="A2" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="B2" s="2" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="C2" s="2" t="n">
+        <v>150</v>
+      </c>
+      <c r="D2" s="4" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="E2" s="2">
+        <f>IF(AND(ISNUMBER(A2),A2&gt;0,ISNUMBER(B2),B2&gt;0,ISNUMBER(C2),C2&gt;=0,ISNUMBER(D2),D2&gt;0,D2&lt;1),A2*B2,"INVALID INPUT")</f>
+        <v/>
+      </c>
+      <c r="F2" s="2">
+        <f>IF(AND(ISNUMBER(A2),A2&gt;0,ISNUMBER(B2),B2&gt;0,ISNUMBER(C2),C2&gt;=0,ISNUMBER(D2),D2&gt;0,D2&lt;1),IF(C2&gt;0,-60*E2*LN(1-D2)/C2,"NO MODELED CLEANING"),"INVALID INPUT")</f>
+        <v/>
+      </c>
+      <c r="G2" s="2">
+        <f>IF(AND(ISNUMBER(A2),A2&gt;0,ISNUMBER(B2),B2&gt;0,ISNUMBER(C2),C2&gt;=0,ISNUMBER(D2),D2&gt;0,D2&lt;1),-2*E2*LN(1-D2),"INVALID INPUT")</f>
+        <v/>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>Illustrative only; no measured D01 CADR</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="68" customHeight="1">
+      <c r="A3" s="3" t="n">
+        <v>25</v>
+      </c>
+      <c r="B3" s="3" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="C3" s="3" t="n">
+        <v>150</v>
+      </c>
+      <c r="D3" s="5" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="E3" s="3">
+        <f>IF(AND(ISNUMBER(A3),A3&gt;0,ISNUMBER(B3),B3&gt;0,ISNUMBER(C3),C3&gt;=0,ISNUMBER(D3),D3&gt;0,D3&lt;1),A3*B3,"INVALID INPUT")</f>
+        <v/>
+      </c>
+      <c r="F3" s="3">
+        <f>IF(AND(ISNUMBER(A3),A3&gt;0,ISNUMBER(B3),B3&gt;0,ISNUMBER(C3),C3&gt;=0,ISNUMBER(D3),D3&gt;0,D3&lt;1),IF(C3&gt;0,-60*E3*LN(1-D3)/C3,"NO MODELED CLEANING"),"INVALID INPUT")</f>
+        <v/>
+      </c>
+      <c r="G3" s="3">
+        <f>IF(AND(ISNUMBER(A3),A3&gt;0,ISNUMBER(B3),B3&gt;0,ISNUMBER(C3),C3&gt;=0,ISNUMBER(D3),D3&gt;0,D3&lt;1),-2*E3*LN(1-D3),"INVALID INPUT")</f>
+        <v/>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>Illustrative only; no measured D01 CADR</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="68" customHeight="1">
+      <c r="A4" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="B4" s="2" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="C4" s="2" t="n">
+        <v>150</v>
+      </c>
+      <c r="D4" s="4" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="E4" s="2">
+        <f>IF(AND(ISNUMBER(A4),A4&gt;0,ISNUMBER(B4),B4&gt;0,ISNUMBER(C4),C4&gt;=0,ISNUMBER(D4),D4&gt;0,D4&lt;1),A4*B4,"INVALID INPUT")</f>
+        <v/>
+      </c>
+      <c r="F4" s="2">
+        <f>IF(AND(ISNUMBER(A4),A4&gt;0,ISNUMBER(B4),B4&gt;0,ISNUMBER(C4),C4&gt;=0,ISNUMBER(D4),D4&gt;0,D4&lt;1),IF(C4&gt;0,-60*E4*LN(1-D4)/C4,"NO MODELED CLEANING"),"INVALID INPUT")</f>
+        <v/>
+      </c>
+      <c r="G4" s="2">
+        <f>IF(AND(ISNUMBER(A4),A4&gt;0,ISNUMBER(B4),B4&gt;0,ISNUMBER(C4),C4&gt;=0,ISNUMBER(D4),D4&gt;0,D4&lt;1),-2*E4*LN(1-D4),"INVALID INPUT")</f>
+        <v/>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>Illustrative only; no measured D01 CADR</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="68" customHeight="1">
+      <c r="A5" s="3" t="n">
+        <v>100</v>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="C5" s="3" t="n">
+        <v>150</v>
+      </c>
+      <c r="D5" s="5" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="E5" s="3">
+        <f>IF(AND(ISNUMBER(A5),A5&gt;0,ISNUMBER(B5),B5&gt;0,ISNUMBER(C5),C5&gt;=0,ISNUMBER(D5),D5&gt;0,D5&lt;1),A5*B5,"INVALID INPUT")</f>
+        <v/>
+      </c>
+      <c r="F5" s="3">
+        <f>IF(AND(ISNUMBER(A5),A5&gt;0,ISNUMBER(B5),B5&gt;0,ISNUMBER(C5),C5&gt;=0,ISNUMBER(D5),D5&gt;0,D5&lt;1),IF(C5&gt;0,-60*E5*LN(1-D5)/C5,"NO MODELED CLEANING"),"INVALID INPUT")</f>
+        <v/>
+      </c>
+      <c r="G5" s="3">
+        <f>IF(AND(ISNUMBER(A5),A5&gt;0,ISNUMBER(B5),B5&gt;0,ISNUMBER(C5),C5&gt;=0,ISNUMBER(D5),D5&gt;0,D5&lt;1),-2*E5*LN(1-D5),"INVALID INPUT")</f>
+        <v/>
+      </c>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>Illustrative only; no measured D01 CADR</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:H5"/>
+  <dataValidations count="4">
+    <dataValidation sqref="A2:A5" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="Invalid scenario" error="Use a positive area/height, nonnegative CADR, and a reduction fraction strictly between0 and1." type="decimal" errorStyle="stop" operator="between">
+      <formula1>0.1</formula1>
+      <formula2>10000</formula2>
+    </dataValidation>
+    <dataValidation sqref="B2:B5" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="Invalid scenario" error="Use a positive area/height, nonnegative CADR, and a reduction fraction strictly between0 and1." type="decimal" errorStyle="stop" operator="between">
+      <formula1>0.1</formula1>
+      <formula2>100</formula2>
+    </dataValidation>
+    <dataValidation sqref="C2:C5" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="Invalid scenario" error="Use a positive area/height, nonnegative CADR, and a reduction fraction strictly between0 and1." type="decimal" errorStyle="stop" operator="between">
+      <formula1>0</formula1>
+      <formula2>100000</formula2>
+    </dataValidation>
+    <dataValidation sqref="D2:D5" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="Invalid scenario" error="Use a positive area/height, nonnegative CADR, and a reduction fraction strictly between0 and1." type="decimal" errorStyle="stop" operator="between">
+      <formula1>1e-06</formula1>
+      <formula2>0.999999</formula2>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A1:M16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>

</xml_diff>

<commit_message>
Complete parallel prototype review batch and refresh handoff bundles
</commit_message>
<xml_diff>
--- a/reports/shareable_20261005/stakeholder/STAKEHOLDER_FUNDING.xlsx
+++ b/reports/shareable_20261005/stakeholder/STAKEHOLDER_FUNDING.xlsx
@@ -14,7 +14,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Funding quotes" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Read me'!$A$1:$B$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Read me'!$A$1:$B$7</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Read me'!$1:$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Milestones'!$A$1:$D$6</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Milestones'!$1:$1</definedName>
@@ -22,7 +22,7 @@
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Claims'!$1:$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Room scenarios'!$A$1:$H$5</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="3">'Room scenarios'!$1:$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Funding quotes'!$A$1:$M$16</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Funding quotes'!$A$1:$M$29</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="4">'Funding quotes'!$1:$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -455,7 +455,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:B7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -474,7 +474,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="36" customHeight="1">
+    <row r="2" ht="38" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Revision</t>
@@ -482,7 +482,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>D01 R03M / IH02 / 5 October 2026</t>
+          <t>D01 R03M / E05 / current parallel batch / 5 October 2026</t>
         </is>
       </c>
     </row>
@@ -498,44 +498,56 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="38" customHeight="1">
+    <row r="4" ht="68" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
+          <t>Current parts</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Funding quotes and Current combined parts use28 current references; other parts/release tabs are historical snapshots. Verify quote unit/kit basis before entering quantity.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="38" customHeight="1">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
           <t>Prices</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="B5" s="3" t="inlineStr">
         <is>
           <t>Blank means UNKNOWN; no prices have been invented.</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="36" customHeight="1">
-      <c r="A5" s="3" t="inlineStr">
+    <row r="6" ht="36" customHeight="1">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>Evidence</t>
         </is>
       </c>
-      <c r="B5" s="3" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>CAD/digital checks are not physical results.</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="38" customHeight="1">
-      <c r="A6" s="2" t="inlineStr">
+    <row r="7" ht="38" customHeight="1">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>Team</t>
         </is>
       </c>
-      <c r="B6" s="2" t="inlineStr">
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>College/NGO funding; no college lab assumed; qualified physical services still needed.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B6"/>
+  <autoFilter ref="A1:B7"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
@@ -1034,19 +1046,19 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:M16"/>
+  <dimension ref="A1:M29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="35.1" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="27.95" customWidth="1" min="2" max="2"/>
+    <col width="17.55" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
     <col width="14" customWidth="1" min="7" max="7"/>
     <col width="14" customWidth="1" min="8" max="8"/>
     <col width="14" customWidth="1" min="9" max="9"/>
-    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="55" customWidth="1" min="10" max="10"/>
     <col width="14" customWidth="1" min="11" max="11"/>
     <col width="22.1" customWidth="1" min="12" max="12"/>
     <col width="55" customWidth="1" min="13" max="13"/>
@@ -1119,7 +1131,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="38" customHeight="1">
+    <row r="2" ht="53" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>F1-F4</t>
@@ -1127,7 +1139,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>ARCTIC P14 Max ACFAN00287A</t>
+          <t>ARCTIC P14 Max black ACFAN00287A</t>
         </is>
       </c>
       <c r="C2" s="2" t="n">
@@ -1139,7 +1151,11 @@
       <c r="G2" s="2" t="inlineStr"/>
       <c r="H2" s="2" t="inlineStr"/>
       <c r="I2" s="2" t="inlineStr"/>
-      <c r="J2" s="2" t="inlineStr"/>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>Delivered revision,cable/connector dimensions,installed duty,guards and protection; quantities are proposals, verify kit/unit basis before quotation</t>
+        </is>
+      </c>
       <c r="K2" s="2" t="inlineStr"/>
       <c r="L2" s="2" t="inlineStr">
         <is>
@@ -1151,7 +1167,7 @@
         <v/>
       </c>
     </row>
-    <row r="3" ht="38" customHeight="1">
+    <row r="3" ht="53" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
           <t>FL1-FL2</t>
@@ -1159,7 +1175,7 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>IKEA STARKVIND104.633.30 particle filter</t>
+          <t>IKEA STARKVIND104.633.30 particle filters</t>
         </is>
       </c>
       <c r="C3" s="3" t="n">
@@ -1171,7 +1187,11 @@
       <c r="G3" s="3" t="inlineStr"/>
       <c r="H3" s="3" t="inlineStr"/>
       <c r="I3" s="3" t="inlineStr"/>
-      <c r="J3" s="3" t="inlineStr"/>
+      <c r="J3" s="3" t="inlineStr">
+        <is>
+          <t>Actual tolerances,frame,seals,clean/loaded resistance; OEM specifies STARKVIND use; quantities are proposals, verify kit/unit basis before quotation</t>
+        </is>
+      </c>
       <c r="K3" s="3" t="inlineStr"/>
       <c r="L3" s="3" t="inlineStr">
         <is>
@@ -1183,7 +1203,7 @@
         <v/>
       </c>
     </row>
-    <row r="4" ht="38" customHeight="1">
+    <row r="4" ht="53" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
           <t>PS1</t>
@@ -1203,7 +1223,11 @@
       <c r="G4" s="2" t="inlineStr"/>
       <c r="H4" s="2" t="inlineStr"/>
       <c r="I4" s="2" t="inlineStr"/>
-      <c r="J4" s="2" t="inlineStr"/>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>Actual startup/auxiliary demand,fault coordination,site suitability; quantities are proposals, verify kit/unit basis before quotation</t>
+        </is>
+      </c>
       <c r="K4" s="2" t="inlineStr"/>
       <c r="L4" s="2" t="inlineStr">
         <is>
@@ -1215,15 +1239,15 @@
         <v/>
       </c>
     </row>
-    <row r="5" ht="38" customHeight="1">
+    <row r="5" ht="53" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>SC1</t>
+          <t>H1</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Noctua NA-FC1</t>
+          <t>Noctua NA-FH1 with supplied NA-EC1</t>
         </is>
       </c>
       <c r="C5" s="3" t="n">
@@ -1235,7 +1259,11 @@
       <c r="G5" s="3" t="inlineStr"/>
       <c r="H5" s="3" t="inlineStr"/>
       <c r="I5" s="3" t="inlineStr"/>
-      <c r="J5" s="3" t="inlineStr"/>
+      <c r="J5" s="3" t="inlineStr">
+        <is>
+          <t>Actual connector fit,retained carrier,cable capacity,abnormal restart behaviour; quantities are proposals, verify kit/unit basis before quotation</t>
+        </is>
+      </c>
       <c r="K5" s="3" t="inlineStr"/>
       <c r="L5" s="3" t="inlineStr">
         <is>
@@ -1247,15 +1275,15 @@
         <v/>
       </c>
     </row>
-    <row r="6" ht="38" customHeight="1">
+    <row r="6" ht="53" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>H1</t>
+          <t>SC1</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Noctua NA-FH1 with NA-EC1</t>
+          <t>Noctua NA-FC1</t>
         </is>
       </c>
       <c r="C6" s="2" t="n">
@@ -1267,7 +1295,11 @@
       <c r="G6" s="2" t="inlineStr"/>
       <c r="H6" s="2" t="inlineStr"/>
       <c r="I6" s="2" t="inlineStr"/>
-      <c r="J6" s="2" t="inlineStr"/>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>Actual mounting,connectors,heat; no live knob interface designed; quantities are proposals, verify kit/unit basis before quotation</t>
+        </is>
+      </c>
       <c r="K6" s="2" t="inlineStr"/>
       <c r="L6" s="2" t="inlineStr">
         <is>
@@ -1279,7 +1311,7 @@
         <v/>
       </c>
     </row>
-    <row r="7" ht="38" customHeight="1">
+    <row r="7" ht="68" customHeight="1">
       <c r="A7" s="3" t="inlineStr">
         <is>
           <t>EXT</t>
@@ -1287,12 +1319,12 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>NA-EC1 300mm from NA-SEC1 kit</t>
+          <t>Noctua NA-EC1 from NA-SEC1 kit</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>2 candidate leads</t>
+          <t>2 candidate extension leads</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr"/>
@@ -1301,7 +1333,11 @@
       <c r="G7" s="3" t="inlineStr"/>
       <c r="H7" s="3" t="inlineStr"/>
       <c r="I7" s="3" t="inlineStr"/>
-      <c r="J7" s="3" t="inlineStr"/>
+      <c r="J7" s="3" t="inlineStr">
+        <is>
+          <t>Exact lead count and connector/gland fit pending;do not duplicate supplied hub lead; quantities are proposals, verify kit/unit basis before quotation</t>
+        </is>
+      </c>
       <c r="K7" s="3" t="inlineStr"/>
       <c r="L7" s="3" t="inlineStr">
         <is>
@@ -1313,21 +1349,19 @@
         <v/>
       </c>
     </row>
-    <row r="8" ht="38" customHeight="1">
+    <row r="8" ht="53" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>CAB</t>
+          <t>CTRL1</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>R03M panels and cleats</t>
-        </is>
-      </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>1 assembly</t>
-        </is>
+          <t>Arduino Opta Lite AFX00003</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="D8" s="2" t="inlineStr"/>
       <c r="E8" s="2" t="inlineStr"/>
@@ -1335,7 +1369,11 @@
       <c r="G8" s="2" t="inlineStr"/>
       <c r="H8" s="2" t="inlineStr"/>
       <c r="I8" s="2" t="inlineStr"/>
-      <c r="J8" s="2" t="inlineStr"/>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>Protective functions not implemented or validated; no upload/physical test; quantities are proposals, verify kit/unit basis before quotation</t>
+        </is>
+      </c>
       <c r="K8" s="2" t="inlineStr"/>
       <c r="L8" s="2" t="inlineStr">
         <is>
@@ -1347,21 +1385,19 @@
         <v/>
       </c>
     </row>
-    <row r="9" ht="38" customHeight="1">
+    <row r="9" ht="53" customHeight="1">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>GUARD</t>
+          <t>CB1</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>R03M welded perforated guards</t>
-        </is>
-      </c>
-      <c r="C9" s="3" t="inlineStr">
-        <is>
-          <t>2 assemblies</t>
-        </is>
+          <t>Hammond1554XA2GY</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="n">
+        <v>1</v>
       </c>
       <c r="D9" s="3" t="inlineStr"/>
       <c r="E9" s="3" t="inlineStr"/>
@@ -1369,7 +1405,11 @@
       <c r="G9" s="3" t="inlineStr"/>
       <c r="H9" s="3" t="inlineStr"/>
       <c r="I9" s="3" t="inlineStr"/>
-      <c r="J9" s="3" t="inlineStr"/>
+      <c r="J9" s="3" t="inlineStr">
+        <is>
+          <t>Whole mounting,entries,thermal,modified ingress,protection and actual fit; quantities are proposals, verify kit/unit basis before quotation</t>
+        </is>
+      </c>
       <c r="K9" s="3" t="inlineStr"/>
       <c r="L9" s="3" t="inlineStr">
         <is>
@@ -1381,21 +1421,19 @@
         <v/>
       </c>
     </row>
-    <row r="10" ht="38" customHeight="1">
+    <row r="10" ht="53" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>FIX</t>
+          <t>PL1</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>R03M fasteners and compression limiters</t>
-        </is>
-      </c>
-      <c r="C10" s="2" t="inlineStr">
-        <is>
-          <t>1 scheduled set</t>
-        </is>
+          <t>Hammond1554XPL</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="D10" s="2" t="inlineStr"/>
       <c r="E10" s="2" t="inlineStr"/>
@@ -1403,7 +1441,11 @@
       <c r="G10" s="2" t="inlineStr"/>
       <c r="H10" s="2" t="inlineStr"/>
       <c r="I10" s="2" t="inlineStr"/>
-      <c r="J10" s="2" t="inlineStr"/>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>Delivered thickness,edge contour,holes,fasteners,functional earth/metal treatment; quantities are proposals, verify kit/unit basis before quotation</t>
+        </is>
+      </c>
       <c r="K10" s="2" t="inlineStr"/>
       <c r="L10" s="2" t="inlineStr">
         <is>
@@ -1415,20 +1457,20 @@
         <v/>
       </c>
     </row>
-    <row r="11" ht="38" customHeight="1">
+    <row r="11" ht="68" customHeight="1">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>SEAL</t>
+          <t>DIN1</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>Filter/fan/penetration seals</t>
+          <t>35x7.5mm rail;Phoenix0801733 reference</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>1 design set</t>
+          <t>1 proposed125mm cut</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr"/>
@@ -1437,7 +1479,11 @@
       <c r="G11" s="3" t="inlineStr"/>
       <c r="H11" s="3" t="inlineStr"/>
       <c r="I11" s="3" t="inlineStr"/>
-      <c r="J11" s="3" t="inlineStr"/>
+      <c r="J11" s="3" t="inlineStr">
+        <is>
+          <t>Obtain suitable cut piece;reference catalogue pack is not procurement quantity;attachment unapproved; quantities are proposals, verify kit/unit basis before quotation</t>
+        </is>
+      </c>
       <c r="K11" s="3" t="inlineStr"/>
       <c r="L11" s="3" t="inlineStr">
         <is>
@@ -1449,19 +1495,19 @@
         <v/>
       </c>
     </row>
-    <row r="12" ht="38" customHeight="1">
+    <row r="12" ht="53" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>FEET</t>
+          <t>PB_START</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Retained feet</t>
+          <t>Schneider ZB5AA3 green spring-return head</t>
         </is>
       </c>
       <c r="C12" s="2" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D12" s="2" t="inlineStr"/>
       <c r="E12" s="2" t="inlineStr"/>
@@ -1469,7 +1515,11 @@
       <c r="G12" s="2" t="inlineStr"/>
       <c r="H12" s="2" t="inlineStr"/>
       <c r="I12" s="2" t="inlineStr"/>
-      <c r="J12" s="2" t="inlineStr"/>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>Actual full stack,labels,torque,retention,sealing; quantities are proposals, verify kit/unit basis before quotation</t>
+        </is>
+      </c>
       <c r="K12" s="2" t="inlineStr"/>
       <c r="L12" s="2" t="inlineStr">
         <is>
@@ -1481,21 +1531,19 @@
         <v/>
       </c>
     </row>
-    <row r="13" ht="38" customHeight="1">
+    <row r="13" ht="53" customHeight="1">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>PR1</t>
+          <t>PB_STOP</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>Protection and service isolation</t>
-        </is>
-      </c>
-      <c r="C13" s="3" t="inlineStr">
-        <is>
-          <t>1 assembly</t>
-        </is>
+          <t>Schneider ZB5AA4 red spring-return head</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="n">
+        <v>1</v>
       </c>
       <c r="D13" s="3" t="inlineStr"/>
       <c r="E13" s="3" t="inlineStr"/>
@@ -1503,7 +1551,11 @@
       <c r="G13" s="3" t="inlineStr"/>
       <c r="H13" s="3" t="inlineStr"/>
       <c r="I13" s="3" t="inlineStr"/>
-      <c r="J13" s="3" t="inlineStr"/>
+      <c r="J13" s="3" t="inlineStr">
+        <is>
+          <t>Not emergency stop,isolation or protective restart; quantities are proposals, verify kit/unit basis before quotation</t>
+        </is>
+      </c>
       <c r="K13" s="3" t="inlineStr"/>
       <c r="L13" s="3" t="inlineStr">
         <is>
@@ -1515,21 +1567,19 @@
         <v/>
       </c>
     </row>
-    <row r="14" ht="38" customHeight="1">
+    <row r="14" ht="53" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>BOX</t>
+          <t>PB_RESET</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Controls enclosure and cable restraints</t>
-        </is>
-      </c>
-      <c r="C14" s="2" t="inlineStr">
-        <is>
-          <t>1 assembly</t>
-        </is>
+          <t>Schneider ZB5AA6 blue spring-return head</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="D14" s="2" t="inlineStr"/>
       <c r="E14" s="2" t="inlineStr"/>
@@ -1537,7 +1587,11 @@
       <c r="G14" s="2" t="inlineStr"/>
       <c r="H14" s="2" t="inlineStr"/>
       <c r="I14" s="2" t="inlineStr"/>
-      <c r="J14" s="2" t="inlineStr"/>
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t>Reset is not start or protective restart approval; quantities are proposals, verify kit/unit basis before quotation</t>
+        </is>
+      </c>
       <c r="K14" s="2" t="inlineStr"/>
       <c r="L14" s="2" t="inlineStr">
         <is>
@@ -1549,21 +1603,19 @@
         <v/>
       </c>
     </row>
-    <row r="15" ht="38" customHeight="1">
+    <row r="15" ht="53" customHeight="1">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>TEST</t>
+          <t>PB_COLLAR</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>Calibrated airflow/pressure/power/noise/PM measurement</t>
-        </is>
-      </c>
-      <c r="C15" s="3" t="inlineStr">
-        <is>
-          <t>1 service scope</t>
-        </is>
+          <t>Schneider ZB5AZ009 fixing collar</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="n">
+        <v>3</v>
       </c>
       <c r="D15" s="3" t="inlineStr"/>
       <c r="E15" s="3" t="inlineStr"/>
@@ -1571,7 +1623,11 @@
       <c r="G15" s="3" t="inlineStr"/>
       <c r="H15" s="3" t="inlineStr"/>
       <c r="I15" s="3" t="inlineStr"/>
-      <c r="J15" s="3" t="inlineStr"/>
+      <c r="J15" s="3" t="inlineStr">
+        <is>
+          <t>Delivered mounting stack and required accessories; quantities are proposals, verify kit/unit basis before quotation</t>
+        </is>
+      </c>
       <c r="K15" s="3" t="inlineStr"/>
       <c r="L15" s="3" t="inlineStr">
         <is>
@@ -1583,21 +1639,19 @@
         <v/>
       </c>
     </row>
-    <row r="16" ht="38" customHeight="1">
+    <row r="16" ht="53" customHeight="1">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>BUILD</t>
+          <t>PB_NO</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Fabrication assembly and qualified review</t>
-        </is>
-      </c>
-      <c r="C16" s="2" t="inlineStr">
-        <is>
-          <t>1 service scope</t>
-        </is>
+          <t>Schneider ZBE1016 gold-flashed NO contact</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="n">
+        <v>2</v>
       </c>
       <c r="D16" s="2" t="inlineStr"/>
       <c r="E16" s="2" t="inlineStr"/>
@@ -1605,7 +1659,11 @@
       <c r="G16" s="2" t="inlineStr"/>
       <c r="H16" s="2" t="inlineStr"/>
       <c r="I16" s="2" t="inlineStr"/>
-      <c r="J16" s="2" t="inlineStr"/>
+      <c r="J16" s="2" t="inlineStr">
+        <is>
+          <t>Numeric minimum switching range,actual terminal identifiers,branch protection; quantities are proposals, verify kit/unit basis before quotation</t>
+        </is>
+      </c>
       <c r="K16" s="2" t="inlineStr"/>
       <c r="L16" s="2" t="inlineStr">
         <is>
@@ -1617,8 +1675,498 @@
         <v/>
       </c>
     </row>
+    <row r="17" ht="53" customHeight="1">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>PB_NC</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>Schneider ZBE1026 gold-flashed NC contact</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D17" s="3" t="inlineStr"/>
+      <c r="E17" s="3" t="inlineStr"/>
+      <c r="F17" s="3" t="inlineStr"/>
+      <c r="G17" s="3" t="inlineStr"/>
+      <c r="H17" s="3" t="inlineStr"/>
+      <c r="I17" s="3" t="inlineStr"/>
+      <c r="J17" s="3" t="inlineStr">
+        <is>
+          <t>Numeric minimum switching range,actual terminal identifiers,branch protection; quantities are proposals, verify kit/unit basis before quotation</t>
+        </is>
+      </c>
+      <c r="K17" s="3" t="inlineStr"/>
+      <c r="L17" s="3" t="inlineStr">
+        <is>
+          <t>UNQUOTED / NOT ORDER AUTHORIZATION</t>
+        </is>
+      </c>
+      <c r="M17" s="3">
+        <f>IF(AND(ISNUMBER(C17),ISNUMBER(F17),ISNUMBER(G17),ISNUMBER(H17)),C17*F17+SUM(G17:H17),"UNQUOTED")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18" ht="68" customHeight="1">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>PR1</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>Independent protection and isolation</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>1 functional assembly</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr"/>
+      <c r="E18" s="2" t="inlineStr"/>
+      <c r="F18" s="2" t="inlineStr"/>
+      <c r="G18" s="2" t="inlineStr"/>
+      <c r="H18" s="2" t="inlineStr"/>
+      <c r="I18" s="2" t="inlineStr"/>
+      <c r="J18" s="2" t="inlineStr">
+        <is>
+          <t>Rated circuit and hazard allocation;ordinary controls/Opta/hub fuse do not substitute; quantities are proposals, verify kit/unit basis before quotation</t>
+        </is>
+      </c>
+      <c r="K18" s="2" t="inlineStr"/>
+      <c r="L18" s="2" t="inlineStr">
+        <is>
+          <t>UNQUOTED / NOT ORDER AUTHORIZATION</t>
+        </is>
+      </c>
+      <c r="M18" s="2">
+        <f>IF(AND(ISNUMBER(C18),ISNUMBER(F18),ISNUMBER(G18),ISNUMBER(H18)),C18*F18+SUM(G18:H18),"UNQUOTED")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19" ht="68" customHeight="1">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>FUSE</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>DC fuse and compatible holder</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>Quantity unknown</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="inlineStr"/>
+      <c r="E19" s="3" t="inlineStr"/>
+      <c r="F19" s="3" t="inlineStr"/>
+      <c r="G19" s="3" t="inlineStr"/>
+      <c r="H19" s="3" t="inlineStr"/>
+      <c r="I19" s="3" t="inlineStr"/>
+      <c r="J19" s="3" t="inlineStr">
+        <is>
+          <t>Fault-time coordination,temperature,contacts and source startup;not a selected fuse; quantities are proposals, verify kit/unit basis before quotation</t>
+        </is>
+      </c>
+      <c r="K19" s="3" t="inlineStr"/>
+      <c r="L19" s="3" t="inlineStr">
+        <is>
+          <t>UNQUOTED / NOT ORDER AUTHORIZATION</t>
+        </is>
+      </c>
+      <c r="M19" s="3">
+        <f>IF(AND(ISNUMBER(C19),ISNUMBER(F19),ISNUMBER(G19),ISNUMBER(H19)),C19*F19+SUM(G19:H19),"UNQUOTED")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20" ht="53" customHeight="1">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>TERM</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>Terminals branch protection and wire system</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>Quantity unknown</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr"/>
+      <c r="E20" s="2" t="inlineStr"/>
+      <c r="F20" s="2" t="inlineStr"/>
+      <c r="G20" s="2" t="inlineStr"/>
+      <c r="H20" s="2" t="inlineStr"/>
+      <c r="I20" s="2" t="inlineStr"/>
+      <c r="J20" s="2" t="inlineStr">
+        <is>
+          <t>Sizes,current/fault/temperature ratings,OEM connectors and label schedule; quantities are proposals, verify kit/unit basis before quotation</t>
+        </is>
+      </c>
+      <c r="K20" s="2" t="inlineStr"/>
+      <c r="L20" s="2" t="inlineStr">
+        <is>
+          <t>UNQUOTED / NOT ORDER AUTHORIZATION</t>
+        </is>
+      </c>
+      <c r="M20" s="2">
+        <f>IF(AND(ISNUMBER(C20),ISNUMBER(F20),ISNUMBER(G20),ISNUMBER(H20)),C20*F20+SUM(G20:H20),"UNQUOTED")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21" ht="53" customHeight="1">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>ENTRY</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>Protected cable entries glands inserts and clamps</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>Quantity unknown</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="inlineStr"/>
+      <c r="E21" s="3" t="inlineStr"/>
+      <c r="F21" s="3" t="inlineStr"/>
+      <c r="G21" s="3" t="inlineStr"/>
+      <c r="H21" s="3" t="inlineStr"/>
+      <c r="I21" s="3" t="inlineStr"/>
+      <c r="J21" s="3" t="inlineStr">
+        <is>
+          <t>Insert size,lead bends,retention,feedthrough seal and guard interface; quantities are proposals, verify kit/unit basis before quotation</t>
+        </is>
+      </c>
+      <c r="K21" s="3" t="inlineStr"/>
+      <c r="L21" s="3" t="inlineStr">
+        <is>
+          <t>UNQUOTED / NOT ORDER AUTHORIZATION</t>
+        </is>
+      </c>
+      <c r="M21" s="3">
+        <f>IF(AND(ISNUMBER(C21),ISNUMBER(F21),ISNUMBER(G21),ISNUMBER(H21)),C21*F21+SUM(G21:H21),"UNQUOTED")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22" ht="53" customHeight="1">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>MOUNT</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>Control box retained mounting and component carriers</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>1 mounting set</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr"/>
+      <c r="E22" s="2" t="inlineStr"/>
+      <c r="F22" s="2" t="inlineStr"/>
+      <c r="G22" s="2" t="inlineStr"/>
+      <c r="H22" s="2" t="inlineStr"/>
+      <c r="I22" s="2" t="inlineStr"/>
+      <c r="J22" s="2" t="inlineStr">
+        <is>
+          <t>Actual support hardware,box placement,tower attachment,service clearance; quantities are proposals, verify kit/unit basis before quotation</t>
+        </is>
+      </c>
+      <c r="K22" s="2" t="inlineStr"/>
+      <c r="L22" s="2" t="inlineStr">
+        <is>
+          <t>UNQUOTED / NOT ORDER AUTHORIZATION</t>
+        </is>
+      </c>
+      <c r="M22" s="2">
+        <f>IF(AND(ISNUMBER(C22),ISNUMBER(F22),ISNUMBER(G22),ISNUMBER(H22)),C22*F22+SUM(G22:H22),"UNQUOTED")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23" ht="53" customHeight="1">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>CAB</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>R03M493-object cabinet geometry</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>1 assembly</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="inlineStr"/>
+      <c r="E23" s="3" t="inlineStr"/>
+      <c r="F23" s="3" t="inlineStr"/>
+      <c r="G23" s="3" t="inlineStr"/>
+      <c r="H23" s="3" t="inlineStr"/>
+      <c r="I23" s="3" t="inlineStr"/>
+      <c r="J23" s="3" t="inlineStr">
+        <is>
+          <t>Material grade,joint strength,whole mass/CG,stability; quantities are proposals, verify kit/unit basis before quotation</t>
+        </is>
+      </c>
+      <c r="K23" s="3" t="inlineStr"/>
+      <c r="L23" s="3" t="inlineStr">
+        <is>
+          <t>UNQUOTED / NOT ORDER AUTHORIZATION</t>
+        </is>
+      </c>
+      <c r="M23" s="3">
+        <f>IF(AND(ISNUMBER(C23),ISNUMBER(F23),ISNUMBER(G23),ISNUMBER(H23)),C23*F23+SUM(G23:H23),"UNQUOTED")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24" ht="53" customHeight="1">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>GUARD</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>R03M perforated guards</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>2 assemblies</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr"/>
+      <c r="E24" s="2" t="inlineStr"/>
+      <c r="F24" s="2" t="inlineStr"/>
+      <c r="G24" s="2" t="inlineStr"/>
+      <c r="H24" s="2" t="inlineStr"/>
+      <c r="I24" s="2" t="inlineStr"/>
+      <c r="J24" s="2" t="inlineStr">
+        <is>
+          <t>Perforated strength,reach,side seam and attachment criteria; quantities are proposals, verify kit/unit basis before quotation</t>
+        </is>
+      </c>
+      <c r="K24" s="2" t="inlineStr"/>
+      <c r="L24" s="2" t="inlineStr">
+        <is>
+          <t>UNQUOTED / NOT ORDER AUTHORIZATION</t>
+        </is>
+      </c>
+      <c r="M24" s="2">
+        <f>IF(AND(ISNUMBER(C24),ISNUMBER(F24),ISNUMBER(G24),ISNUMBER(H24)),C24*F24+SUM(G24:H24),"UNQUOTED")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25" ht="53" customHeight="1">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>FIX</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>R03M fasteners and compression limiters</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>One scheduled set</t>
+        </is>
+      </c>
+      <c r="D25" s="3" t="inlineStr"/>
+      <c r="E25" s="3" t="inlineStr"/>
+      <c r="F25" s="3" t="inlineStr"/>
+      <c r="G25" s="3" t="inlineStr"/>
+      <c r="H25" s="3" t="inlineStr"/>
+      <c r="I25" s="3" t="inlineStr"/>
+      <c r="J25" s="3" t="inlineStr">
+        <is>
+          <t>Actual grades,torques,bearing,withdrawal and tolerances; quantities are proposals, verify kit/unit basis before quotation</t>
+        </is>
+      </c>
+      <c r="K25" s="3" t="inlineStr"/>
+      <c r="L25" s="3" t="inlineStr">
+        <is>
+          <t>UNQUOTED / NOT ORDER AUTHORIZATION</t>
+        </is>
+      </c>
+      <c r="M25" s="3">
+        <f>IF(AND(ISNUMBER(C25),ISNUMBER(F25),ISNUMBER(G25),ISNUMBER(H25)),C25*F25+SUM(G25:H25),"UNQUOTED")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26" ht="53" customHeight="1">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>SEAL</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>Filter fan and penetration gaskets</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>One design set</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr"/>
+      <c r="E26" s="2" t="inlineStr"/>
+      <c r="F26" s="2" t="inlineStr"/>
+      <c r="G26" s="2" t="inlineStr"/>
+      <c r="H26" s="2" t="inlineStr"/>
+      <c r="I26" s="2" t="inlineStr"/>
+      <c r="J26" s="2" t="inlineStr">
+        <is>
+          <t>Force-compression curves,flatness,tolerances,bypass and closure loads; quantities are proposals, verify kit/unit basis before quotation</t>
+        </is>
+      </c>
+      <c r="K26" s="2" t="inlineStr"/>
+      <c r="L26" s="2" t="inlineStr">
+        <is>
+          <t>UNQUOTED / NOT ORDER AUTHORIZATION</t>
+        </is>
+      </c>
+      <c r="M26" s="2">
+        <f>IF(AND(ISNUMBER(C26),ISNUMBER(F26),ISNUMBER(G26),ISNUMBER(H26)),C26*F26+SUM(G26:H26),"UNQUOTED")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27" ht="53" customHeight="1">
+      <c r="A27" s="3" t="inlineStr">
+        <is>
+          <t>FEET</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>R03M retained feet</t>
+        </is>
+      </c>
+      <c r="C27" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="D27" s="3" t="inlineStr"/>
+      <c r="E27" s="3" t="inlineStr"/>
+      <c r="F27" s="3" t="inlineStr"/>
+      <c r="G27" s="3" t="inlineStr"/>
+      <c r="H27" s="3" t="inlineStr"/>
+      <c r="I27" s="3" t="inlineStr"/>
+      <c r="J27" s="3" t="inlineStr">
+        <is>
+          <t>Material,retention,bearing,complete stability and cable-pull evidence; quantities are proposals, verify kit/unit basis before quotation</t>
+        </is>
+      </c>
+      <c r="K27" s="3" t="inlineStr"/>
+      <c r="L27" s="3" t="inlineStr">
+        <is>
+          <t>UNQUOTED / NOT ORDER AUTHORIZATION</t>
+        </is>
+      </c>
+      <c r="M27" s="3">
+        <f>IF(AND(ISNUMBER(C27),ISNUMBER(F27),ISNUMBER(G27),ISNUMBER(H27)),C27*F27+SUM(G27:H27),"UNQUOTED")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28" ht="53" customHeight="1">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>TEST</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>Calibrated airflow pressure power noise PM tests</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>One service scope</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr"/>
+      <c r="E28" s="2" t="inlineStr"/>
+      <c r="F28" s="2" t="inlineStr"/>
+      <c r="G28" s="2" t="inlineStr"/>
+      <c r="H28" s="2" t="inlineStr"/>
+      <c r="I28" s="2" t="inlineStr"/>
+      <c r="J28" s="2" t="inlineStr">
+        <is>
+          <t>Exact methods,instruments,room and acceptance thresholds; quantities are proposals, verify kit/unit basis before quotation</t>
+        </is>
+      </c>
+      <c r="K28" s="2" t="inlineStr"/>
+      <c r="L28" s="2" t="inlineStr">
+        <is>
+          <t>UNQUOTED / NOT ORDER AUTHORIZATION</t>
+        </is>
+      </c>
+      <c r="M28" s="2">
+        <f>IF(AND(ISNUMBER(C28),ISNUMBER(F28),ISNUMBER(G28),ISNUMBER(H28)),C28*F28+SUM(G28:H28),"UNQUOTED")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29" ht="53" customHeight="1">
+      <c r="A29" s="3" t="inlineStr">
+        <is>
+          <t>BUILD</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>Qualified fabrication assembly and commissioning</t>
+        </is>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>One service scope</t>
+        </is>
+      </c>
+      <c r="D29" s="3" t="inlineStr"/>
+      <c r="E29" s="3" t="inlineStr"/>
+      <c r="F29" s="3" t="inlineStr"/>
+      <c r="G29" s="3" t="inlineStr"/>
+      <c r="H29" s="3" t="inlineStr"/>
+      <c r="I29" s="3" t="inlineStr"/>
+      <c r="J29" s="3" t="inlineStr">
+        <is>
+          <t>Real quotes,review scope,procurement authorization and signed physical results; quantities are proposals, verify kit/unit basis before quotation</t>
+        </is>
+      </c>
+      <c r="K29" s="3" t="inlineStr"/>
+      <c r="L29" s="3" t="inlineStr">
+        <is>
+          <t>UNQUOTED / NOT ORDER AUTHORIZATION</t>
+        </is>
+      </c>
+      <c r="M29" s="3">
+        <f>IF(AND(ISNUMBER(C29),ISNUMBER(F29),ISNUMBER(G29),ISNUMBER(H29)),C29*F29+SUM(G29:H29),"UNQUOTED")</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M16"/>
+  <autoFilter ref="A1:M29"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
 </worksheet>

</xml_diff>